<commit_message>
Zmiana progu + kolejna wersja danych :)))
</commit_message>
<xml_diff>
--- a/data/xlsx/KNF_Rejestr_dostawcow_i_wydawcow_pieniadza_elektronicznego.xlsx
+++ b/data/xlsx/KNF_Rejestr_dostawcow_i_wydawcow_pieniadza_elektronicznego.xlsx
@@ -125,12 +125,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2015/17/05</t>
+          <t>2021/10/09</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>11-08-2020</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -192,7 +192,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2022-22-07</t>
+          <t>2020-09-03</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -249,12 +249,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2017-07-03</t>
+          <t>2018-20-04</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>20230905</t>
+          <t>20170321</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -316,7 +316,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16/03/2024</t>
+          <t>24/02/2021</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -378,7 +378,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2023/05/04</t>
+          <t>2020/07/08</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -435,12 +435,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2020/24/10</t>
+          <t>2024/24/06</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>01-01-2025</t>
+          <t>26-05-2023</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2022-12-10</t>
+          <t>2026-17-08</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>16/10/2017</t>
+          <t>10/08/2017</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2023/14/10</t>
+          <t>2022/27/08</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>13-05-2024</t>
+          <t>17-03-2024</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2023-24-01</t>
+          <t>2017-05-10</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -869,12 +869,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2015-17-05</t>
+          <t>2019-27-03</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>20230704</t>
+          <t>20180225</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>20160624</t>
+          <t>20250217</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>03/07/2017</t>
+          <t>26/04/2022</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2018/10/08</t>
+          <t>2026/10/08</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1241,12 +1241,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>20211103</t>
+          <t>20251120</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>25/04/2025</t>
+          <t>21/10/2024</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2025/18/10</t>
+          <t>2017/14/12</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2023/17/01</t>
+          <t>2026/20/07</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2025-20-09</t>
+          <t>2023-03-09</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>27/12/2023</t>
+          <t>23/02/2017</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1613,12 +1613,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>17/05/2015</t>
+          <t>25/04/2022</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2025/09/02</t>
+          <t>2021/26/03</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2022/25/08</t>
+          <t>2025/12/02</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2025-23-05</t>
+          <t>2024-25-04</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2018-08-10</t>
+          <t>2021-18-06</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>20190917</t>
+          <t>20250423</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2021/03/11</t>
+          <t>2026/08/02</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2022-12-03</t>
+          <t>2019-07-03</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>27/09/2020</t>
+          <t>19/06/2018</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>24/06/2025</t>
+          <t>01/08/2026</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>27-10-2024</t>
+          <t>14-12-2017</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2024-08-10</t>
+          <t>2018-09-11</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2016-24-06</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>11/12/2024</t>
+          <t>12/09/2019</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2543,12 +2543,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>10/08/2018</t>
+          <t>07/06/2020</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2020/01/08</t>
+          <t>2019/09/05</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2019/17/09</t>
+          <t>2026/28/09</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>23-12-2022</t>
+          <t>15-04-2026</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>20241018</t>
+          <t>20200130</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>02/02/2019</t>
+          <t>12/08/2018</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>17/01/2023</t>
+          <t>05/11/2026</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2024-22-12</t>
+          <t>2018-01-03</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>20200724</t>
+          <t>20171211</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3101,12 +3101,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>20150517</t>
+          <t>20191002</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>04/08/2025</t>
+          <t>11/01/2018</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>2025/25/01</t>
+          <t>2019/22/02</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2017/03/07</t>
+          <t>2025/11/05</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>25-08-2022</t>
+          <t>10-11-2026</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2019-17-09</t>
+          <t>2024-28-11</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>2024/09/10</t>
+          <t>2017/13/05</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>12-04-2019</t>
+          <t>09-02-2018</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>2024-11-10</t>
+          <t>2018-21-11</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>09/11/2021</t>
+          <t>17/05/2020</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3845,12 +3845,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2015/17/05</t>
+          <t>2018/03/07</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>06-01-2019</t>
+          <t>03-06-2017</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>24-06-2016</t>
+          <t>24-05-2026</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3969,12 +3969,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2017-07-03</t>
+          <t>2025-12-08</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>20250226</t>
+          <t>20240713</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2018-10-08 07:37</t>
+          <t>2025-08-10 07:37</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>2024/16/01</t>
+          <t>2020/27/05</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2020/24/10</t>
+          <t>2026/25/08</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03-11-2021</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>2019/23/07</t>
+          <t>2018/22/04</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>08-12-2022</t>
+          <t>05-06-2022</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>2021-18-03</t>
+          <t>2018-01-02</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4589,12 +4589,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2015-17-05</t>
+          <t>2019-06-11</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>20220126</t>
+          <t>20181007</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4651,12 +4651,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>20160624</t>
+          <t>20210114</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>11/08/2020</t>
+          <t>16/12/2019</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>2024/03/10</t>
+          <t>2024/13/05</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>2024-29-05</t>
+          <t>2017-21-06</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2020-24-10</t>
+          <t>2023-12-12</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>01/03/2019</t>
+          <t>08/01/2019</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>2023/30/06</t>
+          <t>2018/13/01</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>08-02-2023</t>
+          <t>31-05-2021</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>17/05/2015</t>
+          <t>25/02/2023</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -5395,12 +5395,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2016/24/06</t>
+          <t>2018/03/02</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>10-11-2020</t>
+          <t>04-01-2017</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>20200329</t>
+          <t>20190123</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>20190917</t>
+          <t>20250301</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>12-01-2023</t>
+          <t>25-02-2018</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2023-17-01</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>2025/15/09</t>
+          <t>2023/14/12</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>27-11-2022</t>
+          <t>05-02-2017</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>17-05-2015</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -6144,7 +6144,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>20240618</t>
+          <t>20230213</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>22/06/2025</t>
+          <t>04/01/2018</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>19-12-2024</t>
+          <t>24-10-2026</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>20181202</t>
+          <t>20170506</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>07/03/2023</t>
+          <t>12/05/2019</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>2023/02/05</t>
+          <t>2022/31/01</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>20250919</t>
+          <t>20210614</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>24/06/2016</t>
+          <t>27/06/2023</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -6950,7 +6950,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>22-02-2021</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>10/09/2020</t>
+          <t>06/03/2018</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2023/20/07</t>
+          <t>2022/17/10</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7255,12 +7255,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2022/17/03</t>
+          <t>2024/27/04</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>19-10-2023</t>
+          <t>29-03-2023</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>2016-17-12</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7379,7 +7379,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2022-04-07</t>
+          <t>2023-12-08</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>17/05/2020</t>
+          <t>25/04/2017</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2024/05/01</t>
+          <t>2018/08/11</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2023/18/03</t>
+          <t>2025/15/10</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>24-06-2016</t>
+          <t>30-10-2020</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2025-21-08</t>
+          <t>2019-01-10</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7689,12 +7689,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2017-07-03</t>
+          <t>2019-16-09</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>20231211</t>
+          <t>20180817</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>20180810</t>
+          <t>20240109</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>07-07-2021</t>
+          <t>06-09-2020</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7999,7 +7999,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2022-12-10</t>
+          <t>2026-17-01</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -8066,7 +8066,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>09/12/2024</t>
+          <t>25/04/2019</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2024/03/11</t>
+          <t>2022/18/12</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8190,7 +8190,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>09-02-2024</t>
+          <t>25-04-2023</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>20160624</t>
+          <t>20261030</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>03/07/2017</t>
+          <t>23/12/2025</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2018/10/08</t>
+          <t>2020/01/03</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -8557,7 +8557,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>17-09-2019</t>
+          <t>08-05-2026</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>20240319</t>
+          <t>20170224</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8686,7 +8686,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>17/01/2024</t>
+          <t>16/01/2021</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>10-11-2020</t>
+          <t>30-04-2017</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>20220204</t>
+          <t>20250621</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -9053,7 +9053,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>01/03/2022</t>
+          <t>22/05/2023</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -9115,12 +9115,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2016/24/06</t>
+          <t>2021/13/02</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>06-12-2022</t>
+          <t>15-01-2020</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9182,7 +9182,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2020-14-06</t>
+          <t>2017-07-11</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9301,7 +9301,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>20190917</t>
+          <t>20240817</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>12/01/2022</t>
+          <t>13/02/2023</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2023/03/12</t>
+          <t>2025/19/02</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -9492,7 +9492,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2021-17-08</t>
+          <t>2020-11-06</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>20240224</t>
+          <t>20260409</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2019-19-09</t>
+          <t>2018-04-12</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>20170703</t>
+          <t>20250329</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -10045,12 +10045,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>17-09-2019 08:56:36</t>
+          <t>25-06-2022 08:56:36</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>23-09-2023</t>
+          <t>26-05-2021</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10169,7 +10169,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2021-11-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -10231,7 +10231,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>20220916</t>
+          <t>20231004</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>09/12/2024</t>
+          <t>20/12/2026</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -10360,7 +10360,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>24-02-2022</t>
+          <t>28-03-2019</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2025-20-06</t>
+          <t>2023-20-06</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>08/09/2025</t>
+          <t>07/05/2021</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -10603,7 +10603,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>24/06/2016</t>
+          <t>07/10/2024</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -10670,7 +10670,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>24-09-2022</t>
+          <t>05-06-2018</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10789,12 +10789,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2019-17-09</t>
+          <t>2021-14-01</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>20240329</t>
+          <t>20191216</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10856,7 +10856,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>01/07/2024</t>
+          <t>15/05/2019</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>2020/12/03</t>
+          <t>2017/21/06</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2022/10/12</t>
+          <t>2026/14/09</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -11037,7 +11037,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>17-01-2023</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -11099,7 +11099,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2024-24-02</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -11285,12 +11285,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2015/17/05</t>
+          <t>2018/20/10</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>19-07-2020</t>
+          <t>20-09-2017</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -11352,7 +11352,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>2023-05-11</t>
+          <t>2019-01-09</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -11409,12 +11409,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2017-07-03</t>
+          <t>2020-20-01</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>20240615</t>
+          <t>20181221</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -11476,7 +11476,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>04/12/2025</t>
+          <t>29/10/2017</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -11533,12 +11533,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>17/09/2019</t>
+          <t>25/08/2021</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>2022/01/07</t>
+          <t>2020/26/07</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -11781,12 +11781,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>20230117</t>
+          <t>20250429</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>16/05/2025</t>
+          <t>30/03/2024</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>20220830</t>
+          <t>20170705</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12091,7 +12091,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>20160624</t>
+          <t>20200828</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -12153,7 +12153,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>03/07/2017</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -12215,12 +12215,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2018/10/08</t>
+          <t>2021/20/04</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>05-04-2024</t>
+          <t>21-03-2020</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -12282,7 +12282,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>2024-25-12</t>
+          <t>2017-02-01</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -12344,7 +12344,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>20240515</t>
+          <t>20230207</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>15/06/2025</t>
+          <t>24/02/2021</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">

</xml_diff>